<commit_message>
Updated scripts for Mexico, for 2025
</commit_message>
<xml_diff>
--- a/regions_Mexico/data/Mortalidad_09.xlsx
+++ b/regions_Mexico/data/Mortalidad_09.xlsx
@@ -5,21 +5,21 @@
     <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Tabulado" sheetId="1" r:id="R2e879ef0f3664098"/>
+    <sheet name="Tabulado" sheetId="1" r:id="Re15587e4ae47444c"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t>Instituto Nacional de Estadística y Geografía (INEGI)</t>
   </si>
   <si>
-    <t>Esperanza de vida al nacimiento por entidad federativa según sexo, serie anual de 2010 a 2025</t>
-  </si>
-  <si>
-    <t>Fecha de consulta: 02/09/2025 17:44:59</t>
+    <t>Esperanza de vida al nacimiento por entidad federativa según sexo, serie anual de 2010 a 2026</t>
+  </si>
+  <si>
+    <t>Fecha de consulta: 27/02/2026 15:12:58</t>
   </si>
   <si>
     <t/>
@@ -79,6 +79,9 @@
     <t>2025</t>
   </si>
   <si>
+    <t>2026</t>
+  </si>
+  <si>
     <t>Total</t>
   </si>
   <si>
@@ -199,16 +202,10 @@
     <t>Número de años que en promedio se espera viva una persona al momento de su nacimiento, suponiendo que la tendencia de la mortalidad no variara, ya que el cálculo de este indicador toma como base las tasas de mortalidad para un determinado año.</t>
   </si>
   <si>
-    <t>Nota:</t>
-  </si>
-  <si>
-    <t>El 12 de septiembre de 2023 se actualizaron los datos correspondientes al período de 2010 a 2023. Esta actualización se deriva de los resultados de la Conciliación Demográfica de 1950 a 2019 y las Proyecciones de la Población de México para el período 2020 a 2070, por parte del Consejo Nacional de Población (CONAPO) publicados el 4 de agosto de 2023.</t>
-  </si>
-  <si>
-    <t>Fuente:</t>
-  </si>
-  <si>
-    <t>CONAPO. Consejo Nacional de Población. Conciliación Demográfica de 1950 a 2019 y Proyecciones de la población de México y de las entidades federativas 2020 a 2070. https://www.gob.mx/conapo/documentos/bases-de-datos-de-la-conciliacion-demografica-1950-a-2019-y-proyecciones-de-la-poblacion-de-mexico-2020-a-2070 (Consulta: 06 de enero de 2025).</t>
+    <t>Fuente: CONAPO. Consejo Nacional de Población. Conciliación Demográfica de 1950 a 2019 y Proyecciones de la población de México y de las entidades federativas 2020 a 2070. https://www.gob.mx/conapo/documentos/bases-de-datos-de-la-conciliacion-demografica-1950-a-2019-y-proyecciones-de-la-poblacion-de-mexico-2020-a-2070 (Consulta: 07 de enero de 2026).</t>
+  </si>
+  <si>
+    <t>Fecha de actualización: 09 de enero de 2026.</t>
   </si>
 </sst>
 </file>
@@ -327,7 +324,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AW55"/>
+  <dimension ref="A1:AZ53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1" style="1"/>
@@ -379,6 +376,9 @@
     <col min="47" max="47" width="20" customWidth="1" style="1"/>
     <col min="48" max="48" width="20" customWidth="1" style="1"/>
     <col min="49" max="49" width="20" customWidth="1" style="1"/>
+    <col min="50" max="50" width="20" customWidth="1" style="1"/>
+    <col min="51" max="51" width="20" customWidth="1" style="1"/>
+    <col min="52" max="52" width="20" customWidth="1" style="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -554,159 +554,177 @@
       <c r="AW7" s="7" t="s">
         <v>21</v>
       </c>
+      <c r="AX7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="AY7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="AZ7" s="7" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="F8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="7" t="s">
+      <c r="G8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="I8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" s="7" t="s">
+      <c r="J8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="L8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="K8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" s="7" t="s">
+      <c r="M8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="N8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="M8" s="7" t="s">
+      <c r="O8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="N8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="O8" s="7" t="s">
+      <c r="P8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="P8" s="7" t="s">
+      <c r="R8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="Q8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R8" s="7" t="s">
+      <c r="S8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="T8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="S8" s="7" t="s">
+      <c r="U8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="T8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="U8" s="7" t="s">
+      <c r="V8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="W8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="V8" s="7" t="s">
+      <c r="X8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="W8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="X8" s="7" t="s">
+      <c r="Y8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="Y8" s="7" t="s">
+      <c r="AA8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="Z8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AA8" s="7" t="s">
+      <c r="AB8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AC8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AB8" s="7" t="s">
+      <c r="AD8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AC8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AD8" s="7" t="s">
+      <c r="AE8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AF8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AE8" s="7" t="s">
+      <c r="AG8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AF8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AG8" s="7" t="s">
+      <c r="AH8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AI8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AH8" s="7" t="s">
+      <c r="AJ8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AI8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AJ8" s="7" t="s">
+      <c r="AK8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AL8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AK8" s="7" t="s">
+      <c r="AM8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AL8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AM8" s="7" t="s">
+      <c r="AN8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AO8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AN8" s="7" t="s">
+      <c r="AP8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AO8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AP8" s="7" t="s">
+      <c r="AQ8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AR8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AQ8" s="7" t="s">
+      <c r="AS8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AR8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AS8" s="7" t="s">
+      <c r="AT8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AU8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AT8" s="7" t="s">
+      <c r="AV8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AU8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AV8" s="7" t="s">
+      <c r="AW8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AX8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AW8" s="7" t="s">
+      <c r="AY8" s="7" t="s">
         <v>24</v>
+      </c>
+      <c r="AZ8" s="7" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9" s="8">
         <v>74.3</v>
@@ -851,11 +869,20 @@
       </c>
       <c r="AW9" s="8">
         <v>79</v>
+      </c>
+      <c r="AX9" s="8">
+        <v>75.9</v>
+      </c>
+      <c r="AY9" s="8">
+        <v>72.7</v>
+      </c>
+      <c r="AZ9" s="8">
+        <v>79.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="9">
         <v>75.7</v>
@@ -1000,11 +1027,20 @@
       </c>
       <c r="AW10" s="9">
         <v>80.3</v>
+      </c>
+      <c r="AX10" s="9">
+        <v>77.2</v>
+      </c>
+      <c r="AY10" s="9">
+        <v>74.2</v>
+      </c>
+      <c r="AZ10" s="9">
+        <v>80.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11" s="8">
         <v>75</v>
@@ -1149,11 +1185,20 @@
       </c>
       <c r="AW11" s="8">
         <v>80</v>
+      </c>
+      <c r="AX11" s="8">
+        <v>76.9</v>
+      </c>
+      <c r="AY11" s="8">
+        <v>73.9</v>
+      </c>
+      <c r="AZ11" s="8">
+        <v>80.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B12" s="9">
         <v>76.2</v>
@@ -1298,11 +1343,20 @@
       </c>
       <c r="AW12" s="9">
         <v>80.5</v>
+      </c>
+      <c r="AX12" s="9">
+        <v>77.5</v>
+      </c>
+      <c r="AY12" s="9">
+        <v>74.6</v>
+      </c>
+      <c r="AZ12" s="9">
+        <v>80.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B13" s="8">
         <v>74.4</v>
@@ -1447,11 +1501,20 @@
       </c>
       <c r="AW13" s="8">
         <v>78.1</v>
+      </c>
+      <c r="AX13" s="8">
+        <v>74.9</v>
+      </c>
+      <c r="AY13" s="8">
+        <v>71.8</v>
+      </c>
+      <c r="AZ13" s="8">
+        <v>78.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="9">
         <v>76.5</v>
@@ -1596,11 +1659,20 @@
       </c>
       <c r="AW14" s="9">
         <v>80.5</v>
+      </c>
+      <c r="AX14" s="9">
+        <v>77.4</v>
+      </c>
+      <c r="AY14" s="9">
+        <v>74.5</v>
+      </c>
+      <c r="AZ14" s="9">
+        <v>80.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15" s="8">
         <v>75.5</v>
@@ -1745,11 +1817,20 @@
       </c>
       <c r="AW15" s="8">
         <v>79.6</v>
+      </c>
+      <c r="AX15" s="8">
+        <v>76.5</v>
+      </c>
+      <c r="AY15" s="8">
+        <v>73.5</v>
+      </c>
+      <c r="AZ15" s="8">
+        <v>79.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B16" s="9">
         <v>72</v>
@@ -1894,11 +1975,20 @@
       </c>
       <c r="AW16" s="9">
         <v>76.6</v>
+      </c>
+      <c r="AX16" s="9">
+        <v>73.4</v>
+      </c>
+      <c r="AY16" s="9">
+        <v>70.3</v>
+      </c>
+      <c r="AZ16" s="9">
+        <v>76.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="8">
         <v>75.2</v>
@@ -2043,11 +2133,20 @@
       </c>
       <c r="AW17" s="8">
         <v>80</v>
+      </c>
+      <c r="AX17" s="8">
+        <v>77</v>
+      </c>
+      <c r="AY17" s="8">
+        <v>74</v>
+      </c>
+      <c r="AZ17" s="8">
+        <v>80.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18" s="9">
         <v>76.3</v>
@@ -2192,11 +2291,20 @@
       </c>
       <c r="AW18" s="9">
         <v>80.2</v>
+      </c>
+      <c r="AX18" s="9">
+        <v>77.2</v>
+      </c>
+      <c r="AY18" s="9">
+        <v>74.2</v>
+      </c>
+      <c r="AZ18" s="9">
+        <v>80.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="8">
         <v>74.1</v>
@@ -2341,11 +2449,20 @@
       </c>
       <c r="AW19" s="8">
         <v>79</v>
+      </c>
+      <c r="AX19" s="8">
+        <v>75.9</v>
+      </c>
+      <c r="AY19" s="8">
+        <v>72.9</v>
+      </c>
+      <c r="AZ19" s="8">
+        <v>79.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B20" s="9">
         <v>73.9</v>
@@ -2490,11 +2607,20 @@
       </c>
       <c r="AW20" s="9">
         <v>78.4</v>
+      </c>
+      <c r="AX20" s="9">
+        <v>75.3</v>
+      </c>
+      <c r="AY20" s="9">
+        <v>72.2</v>
+      </c>
+      <c r="AZ20" s="9">
+        <v>78.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B21" s="8">
         <v>72.3</v>
@@ -2639,11 +2765,20 @@
       </c>
       <c r="AW21" s="8">
         <v>76.8</v>
+      </c>
+      <c r="AX21" s="8">
+        <v>73.5</v>
+      </c>
+      <c r="AY21" s="8">
+        <v>70.4</v>
+      </c>
+      <c r="AZ21" s="8">
+        <v>77</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B22" s="9">
         <v>73.4</v>
@@ -2788,11 +2923,20 @@
       </c>
       <c r="AW22" s="9">
         <v>77.5</v>
+      </c>
+      <c r="AX22" s="9">
+        <v>74.3</v>
+      </c>
+      <c r="AY22" s="9">
+        <v>71.2</v>
+      </c>
+      <c r="AZ22" s="9">
+        <v>77.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B23" s="8">
         <v>74.8</v>
@@ -2937,11 +3081,20 @@
       </c>
       <c r="AW23" s="8">
         <v>79.5</v>
+      </c>
+      <c r="AX23" s="8">
+        <v>76.4</v>
+      </c>
+      <c r="AY23" s="8">
+        <v>73.4</v>
+      </c>
+      <c r="AZ23" s="8">
+        <v>79.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B24" s="9">
         <v>74.3</v>
@@ -3086,11 +3239,20 @@
       </c>
       <c r="AW24" s="9">
         <v>78.6</v>
+      </c>
+      <c r="AX24" s="9">
+        <v>75.5</v>
+      </c>
+      <c r="AY24" s="9">
+        <v>72.5</v>
+      </c>
+      <c r="AZ24" s="9">
+        <v>78.8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B25" s="8">
         <v>73.1</v>
@@ -3235,11 +3397,20 @@
       </c>
       <c r="AW25" s="8">
         <v>77.7</v>
+      </c>
+      <c r="AX25" s="8">
+        <v>74.5</v>
+      </c>
+      <c r="AY25" s="8">
+        <v>71.4</v>
+      </c>
+      <c r="AZ25" s="8">
+        <v>78</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B26" s="9">
         <v>73.9</v>
@@ -3384,11 +3555,20 @@
       </c>
       <c r="AW26" s="9">
         <v>77.9</v>
+      </c>
+      <c r="AX26" s="9">
+        <v>74.7</v>
+      </c>
+      <c r="AY26" s="9">
+        <v>71.6</v>
+      </c>
+      <c r="AZ26" s="9">
+        <v>78.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B27" s="8">
         <v>74.4</v>
@@ -3533,11 +3713,20 @@
       </c>
       <c r="AW27" s="8">
         <v>79.1</v>
+      </c>
+      <c r="AX27" s="8">
+        <v>76</v>
+      </c>
+      <c r="AY27" s="8">
+        <v>72.9</v>
+      </c>
+      <c r="AZ27" s="8">
+        <v>79.3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B28" s="9">
         <v>77.4</v>
@@ -3682,11 +3871,20 @@
       </c>
       <c r="AW28" s="9">
         <v>81.1</v>
+      </c>
+      <c r="AX28" s="9">
+        <v>78.1</v>
+      </c>
+      <c r="AY28" s="9">
+        <v>75.1</v>
+      </c>
+      <c r="AZ28" s="9">
+        <v>81.3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B29" s="8">
         <v>72.7</v>
@@ -3831,11 +4029,20 @@
       </c>
       <c r="AW29" s="8">
         <v>77</v>
+      </c>
+      <c r="AX29" s="8">
+        <v>73.7</v>
+      </c>
+      <c r="AY29" s="8">
+        <v>70.5</v>
+      </c>
+      <c r="AZ29" s="8">
+        <v>77.2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B30" s="9">
         <v>73</v>
@@ -3980,11 +4187,20 @@
       </c>
       <c r="AW30" s="9">
         <v>77.5</v>
+      </c>
+      <c r="AX30" s="9">
+        <v>74.3</v>
+      </c>
+      <c r="AY30" s="9">
+        <v>71.2</v>
+      </c>
+      <c r="AZ30" s="9">
+        <v>77.7</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B31" s="8">
         <v>74.7</v>
@@ -4129,11 +4345,20 @@
       </c>
       <c r="AW31" s="8">
         <v>79.7</v>
+      </c>
+      <c r="AX31" s="8">
+        <v>76.6</v>
+      </c>
+      <c r="AY31" s="8">
+        <v>73.6</v>
+      </c>
+      <c r="AZ31" s="8">
+        <v>79.9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B32" s="9">
         <v>75.1</v>
@@ -4278,11 +4503,20 @@
       </c>
       <c r="AW32" s="9">
         <v>79.4</v>
+      </c>
+      <c r="AX32" s="9">
+        <v>76.4</v>
+      </c>
+      <c r="AY32" s="9">
+        <v>73.4</v>
+      </c>
+      <c r="AZ32" s="9">
+        <v>79.6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B33" s="8">
         <v>74.2</v>
@@ -4427,11 +4661,20 @@
       </c>
       <c r="AW33" s="8">
         <v>78.8</v>
+      </c>
+      <c r="AX33" s="8">
+        <v>75.7</v>
+      </c>
+      <c r="AY33" s="8">
+        <v>72.6</v>
+      </c>
+      <c r="AZ33" s="8">
+        <v>79</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B34" s="9">
         <v>74.7</v>
@@ -4576,11 +4819,20 @@
       </c>
       <c r="AW34" s="9">
         <v>79.5</v>
+      </c>
+      <c r="AX34" s="9">
+        <v>76.5</v>
+      </c>
+      <c r="AY34" s="9">
+        <v>73.5</v>
+      </c>
+      <c r="AZ34" s="9">
+        <v>79.7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B35" s="8">
         <v>75.6</v>
@@ -4725,11 +4977,20 @@
       </c>
       <c r="AW35" s="8">
         <v>80.1</v>
+      </c>
+      <c r="AX35" s="8">
+        <v>77.1</v>
+      </c>
+      <c r="AY35" s="8">
+        <v>74.1</v>
+      </c>
+      <c r="AZ35" s="8">
+        <v>80.3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B36" s="9">
         <v>72.9</v>
@@ -4874,11 +5135,20 @@
       </c>
       <c r="AW36" s="9">
         <v>77.4</v>
+      </c>
+      <c r="AX36" s="9">
+        <v>74.2</v>
+      </c>
+      <c r="AY36" s="9">
+        <v>71.1</v>
+      </c>
+      <c r="AZ36" s="9">
+        <v>77.6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B37" s="8">
         <v>75.1</v>
@@ -5023,11 +5293,20 @@
       </c>
       <c r="AW37" s="8">
         <v>79.3</v>
+      </c>
+      <c r="AX37" s="8">
+        <v>76.2</v>
+      </c>
+      <c r="AY37" s="8">
+        <v>73.2</v>
+      </c>
+      <c r="AZ37" s="8">
+        <v>79.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B38" s="9">
         <v>73.2</v>
@@ -5172,11 +5451,20 @@
       </c>
       <c r="AW38" s="9">
         <v>77.8</v>
+      </c>
+      <c r="AX38" s="9">
+        <v>74.6</v>
+      </c>
+      <c r="AY38" s="9">
+        <v>71.5</v>
+      </c>
+      <c r="AZ38" s="9">
+        <v>78</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B39" s="8">
         <v>73.4</v>
@@ -5321,11 +5609,20 @@
       </c>
       <c r="AW39" s="8">
         <v>77.3</v>
+      </c>
+      <c r="AX39" s="8">
+        <v>74.1</v>
+      </c>
+      <c r="AY39" s="8">
+        <v>71</v>
+      </c>
+      <c r="AZ39" s="8">
+        <v>77.6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B40" s="9">
         <v>74.2</v>
@@ -5470,11 +5767,20 @@
       </c>
       <c r="AW40" s="9">
         <v>78.5</v>
+      </c>
+      <c r="AX40" s="9">
+        <v>75.4</v>
+      </c>
+      <c r="AY40" s="9">
+        <v>72.3</v>
+      </c>
+      <c r="AZ40" s="9">
+        <v>78.7</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B41" s="8">
         <v>73.4</v>
@@ -5619,16 +5925,25 @@
       </c>
       <c r="AW41" s="8">
         <v>78</v>
+      </c>
+      <c r="AX41" s="8">
+        <v>74.8</v>
+      </c>
+      <c r="AY41" s="8">
+        <v>71.6</v>
+      </c>
+      <c r="AZ41" s="8">
+        <v>78.2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="46">
@@ -5638,12 +5953,12 @@
     </row>
     <row r="47">
       <c r="A47" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49">
@@ -5653,31 +5968,21 @@
     </row>
     <row r="50">
       <c r="A50" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="s">
-        <v>63</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="s">
-        <v>3</v>
+        <v>64</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="s">
+      <c r="A53" s="4" t="s">
         <v>3</v>
       </c>
     </row>
@@ -5699,6 +6004,7 @@
     <mergeCell ref="AO7:AQ7"/>
     <mergeCell ref="AR7:AT7"/>
     <mergeCell ref="AU7:AW7"/>
+    <mergeCell ref="AX7:AZ7"/>
     <mergeCell ref="A7:A8"/>
   </mergeCells>
   <headerFooter/>

</xml_diff>